<commit_message>
Update billing system files and build outputs
</commit_message>
<xml_diff>
--- a/inventory_billing.xlsx
+++ b/inventory_billing.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -483,17 +483,38 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Mouse</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>340</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>10101010</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
         <v>5</v>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>Pencil</t>
         </is>
       </c>
-      <c r="C4" t="n">
+      <c r="C5" t="n">
         <v>20</v>
       </c>
-      <c r="E4" t="n">
+      <c r="E5" t="n">
         <v>30</v>
       </c>
     </row>
@@ -508,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -565,153 +586,191 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Bipana</t>
+          <t>Umanga</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>9812345076</t>
+          <t>981298474398</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-09-16 16:09:10</t>
+          <t>2026-09-16 21:50:18</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>1400</v>
+        <v>18700</v>
       </c>
       <c r="F2" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G2" t="n">
-        <v>84</v>
+        <v>561</v>
       </c>
       <c r="H2" t="n">
         <v>13</v>
       </c>
       <c r="I2" t="n">
-        <v>171.08</v>
+        <v>2358.07</v>
       </c>
       <c r="J2" t="n">
-        <v>1487.08</v>
+        <v>20497.07</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Kabya</t>
+          <t>Bipana</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>9876543210</t>
+          <t>9812345076</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-09-16 15:59:01</t>
+          <t>2026-09-16 16:09:10</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>750</v>
+        <v>1400</v>
       </c>
       <c r="F3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G3" t="n">
-        <v>37.5</v>
+        <v>84</v>
       </c>
       <c r="H3" t="n">
         <v>13</v>
       </c>
       <c r="I3" t="n">
-        <v>92.625</v>
+        <v>171.08</v>
       </c>
       <c r="J3" t="n">
-        <v>805.125</v>
+        <v>1487.08</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Priyanshu</t>
+          <t>Kabya</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>986218230438</t>
+          <t>9876543210</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-09-16 15:51:46</t>
+          <t>2026-09-16 15:59:01</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>4500</v>
+        <v>750</v>
       </c>
       <c r="F4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G4" t="n">
-        <v>180</v>
+        <v>37.5</v>
       </c>
       <c r="H4" t="n">
         <v>13</v>
       </c>
       <c r="I4" t="n">
-        <v>561.6</v>
+        <v>92.625</v>
       </c>
       <c r="J4" t="n">
-        <v>4881.6</v>
+        <v>805.125</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Serab</t>
+          <t>Priyanshu</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>9812345678</t>
+          <t>986218230438</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-07-30 16:37:50</t>
+          <t>2026-09-16 15:51:46</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>60000</v>
+        <v>4500</v>
       </c>
       <c r="F5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G5" t="n">
-        <v>3000</v>
+        <v>180</v>
       </c>
       <c r="H5" t="n">
         <v>13</v>
       </c>
       <c r="I5" t="n">
+        <v>561.6</v>
+      </c>
+      <c r="J5" t="n">
+        <v>4881.6</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Serab</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>9812345678</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2026-07-30 16:37:50</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>60000</v>
+      </c>
+      <c r="F6" t="n">
+        <v>5</v>
+      </c>
+      <c r="G6" t="n">
+        <v>3000</v>
+      </c>
+      <c r="H6" t="n">
+        <v>13</v>
+      </c>
+      <c r="I6" t="n">
         <v>7410</v>
       </c>
-      <c r="J5" t="n">
+      <c r="J6" t="n">
         <v>64410</v>
       </c>
     </row>

</xml_diff>